<commit_message>
feat(template): add Asesmen column (UK1-UK5) to CPMK sheet in import template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apsi2026/public/templates/Template_Import_SICPL_KOSONG.xlsx
+++ b/apsi2026/public/templates/Template_Import_SICPL_KOSONG.xlsx
@@ -844,12 +844,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>CPMK milik 1 Mata Kuliah. Deskripsi Inggris opsional tapi disarankan.</v>
       </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -864,6 +867,9 @@
       <c r="D2" t="str">
         <v>Deskripsi (English)</v>
       </c>
+      <c r="E2" t="str">
+        <v>Asesmen</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -877,6 +883,9 @@
       </c>
       <c r="D3" t="str">
         <v>Analyze user requirements.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>UK1</v>
       </c>
     </row>
   </sheetData>
@@ -885,7 +894,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>